<commit_message>
new changes to readme file
</commit_message>
<xml_diff>
--- a/CSO_prediction/comparison_methods/comparison.xlsx
+++ b/CSO_prediction/comparison_methods/comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/mr861_exeter_ac_uk/Documents/Desktop/model_Faf/CSO_prediction/comparison_methods/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_F25DC773A252ABDACC10484C319C55345ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8256FE2-7D86-42B7-B467-DE0A2B259705}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="11_F25DC773A252ABDACC10484C319C55345ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFA5075F-C2FA-416D-AC90-15A39A29174D}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="13">
   <si>
     <t xml:space="preserve">peak flow error </t>
   </si>
@@ -53,13 +53,28 @@
     <t>max_observed</t>
   </si>
   <si>
-    <t>Peak Erro (%)</t>
-  </si>
-  <si>
     <t>LSTM</t>
   </si>
   <si>
     <t>XGBoost</t>
+  </si>
+  <si>
+    <t>GPR (constrained)</t>
+  </si>
+  <si>
+    <t>RMSE</t>
+  </si>
+  <si>
+    <t>GPR (mean)</t>
+  </si>
+  <si>
+    <t>GPR (kernel)</t>
+  </si>
+  <si>
+    <t>GPR (naïve)</t>
+  </si>
+  <si>
+    <t>Peak Error (%)</t>
   </si>
 </sst>
 </file>
@@ -131,6 +146,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -396,42 +415,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.23046875" style="1"/>
-    <col min="3" max="3" width="13.4609375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.15234375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="19.61328125" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.23046875" style="1"/>
+    <col min="1" max="1" width="25" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" style="1"/>
+    <col min="3" max="3" width="13.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" style="1" customWidth="1"/>
+    <col min="6" max="8" width="9.21875" style="1"/>
+    <col min="9" max="9" width="18.109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="9.21875" style="1"/>
+    <col min="11" max="12" width="13.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="16.33203125" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.21875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="B4" s="1">
         <v>2021</v>
@@ -446,13 +491,203 @@
         <f>100*(D4-C4)/D4</f>
         <v>70.960460118550159</v>
       </c>
+      <c r="F4" s="1">
+        <v>77.816100000000006</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="1">
+        <v>2019</v>
+      </c>
+      <c r="K4" s="1">
+        <v>125.3497</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="N4" s="1">
+        <v>12.706799999999999</v>
+      </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="B5" s="1">
         <v>2021</v>
+      </c>
+      <c r="C5" s="1">
+        <v>502.95190000000002</v>
+      </c>
+      <c r="D5" s="1">
+        <v>939.63610000000006</v>
+      </c>
+      <c r="E5" s="1">
+        <f>100*(D5-C5)/D5</f>
+        <v>46.473757234316565</v>
+      </c>
+      <c r="F5" s="1">
+        <v>46.997300000000003</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="1">
+        <v>2019</v>
+      </c>
+      <c r="K5" s="1">
+        <v>316.32420000000002</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="N5" s="1">
+        <v>14.6439</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2021</v>
+      </c>
+      <c r="C6" s="1">
+        <v>456.09710000000001</v>
+      </c>
+      <c r="D6" s="1">
+        <v>939.63610000000006</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" ref="E6:E9" si="0">100*(D6-C6)/D6</f>
+        <v>51.46024083153042</v>
+      </c>
+      <c r="F6" s="1">
+        <v>98.424999999999997</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="1">
+        <v>2019</v>
+      </c>
+      <c r="K6" s="1">
+        <v>232.1156</v>
+      </c>
+      <c r="L6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6" s="1">
+        <v>40.370399999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2021</v>
+      </c>
+      <c r="C7" s="1">
+        <v>456.02859999999998</v>
+      </c>
+      <c r="D7" s="1">
+        <v>939.63610000000006</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>51.46753088775538</v>
+      </c>
+      <c r="F7" s="1">
+        <v>105.8365</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" s="1">
+        <v>2019</v>
+      </c>
+      <c r="K7" s="1">
+        <v>229.93020000000001</v>
+      </c>
+      <c r="L7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>24.8491</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2021</v>
+      </c>
+      <c r="C8" s="1">
+        <v>451.20100000000002</v>
+      </c>
+      <c r="D8" s="1">
+        <v>939.63610000000006</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>51.981304251720424</v>
+      </c>
+      <c r="F8" s="1">
+        <v>105.7893</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="1">
+        <v>2019</v>
+      </c>
+      <c r="K8" s="1">
+        <v>229.81219999999999</v>
+      </c>
+      <c r="L8" s="1">
+        <v>0</v>
+      </c>
+      <c r="N8" s="1">
+        <v>24.807500000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2021</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0</v>
+      </c>
+      <c r="D9" s="1">
+        <v>939.63610000000006</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="F9" s="1">
+        <v>102.62</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="1">
+        <v>2019</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1">
+        <v>0</v>
+      </c>
+      <c r="N9" s="1">
+        <v>127.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>